<commit_message>
replace gmail smtp with resend email api
</commit_message>
<xml_diff>
--- a/backend/exports/enquiries.xlsx
+++ b/backend/exports/enquiries.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="93">
   <si>
     <t>S.No</t>
   </si>
@@ -248,6 +248,48 @@
   </si>
   <si>
     <t>7/6/2026, 12:15:29 am</t>
+  </si>
+  <si>
+    <t>simple</t>
+  </si>
+  <si>
+    <t>simple@gmail.com</t>
+  </si>
+  <si>
+    <t>9847548657</t>
+  </si>
+  <si>
+    <t>test final</t>
+  </si>
+  <si>
+    <t>7/6/2026, 12:19:18 am</t>
+  </si>
+  <si>
+    <t>random</t>
+  </si>
+  <si>
+    <t>random@gmail.com</t>
+  </si>
+  <si>
+    <t>9845748654</t>
+  </si>
+  <si>
+    <t>Cloud Computing</t>
+  </si>
+  <si>
+    <t>test 004</t>
+  </si>
+  <si>
+    <t>7/6/2026, 12:27:20 am</t>
+  </si>
+  <si>
+    <t>Arudra Siva Sai Sunkari</t>
+  </si>
+  <si>
+    <t>arudrasunkari18@gmail.com</t>
+  </si>
+  <si>
+    <t>7/6/2026, 12:38:23 am</t>
   </si>
 </sst>
 </file>
@@ -634,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1096,6 +1138,102 @@
         <v>78</v>
       </c>
     </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>82</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" t="s">
+        <v>24</v>
+      </c>
+      <c r="J15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" t="s">
+        <v>87</v>
+      </c>
+      <c r="F16" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" t="s">
+        <v>51</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" t="s">
+        <v>17</v>
+      </c>
+      <c r="J17" t="s">
+        <v>92</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
added resend for mail sending
</commit_message>
<xml_diff>
--- a/backend/exports/enquiries.xlsx
+++ b/backend/exports/enquiries.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="103">
   <si>
     <t>S.No</t>
   </si>
@@ -290,6 +290,36 @@
   </si>
   <si>
     <t>7/6/2026, 12:38:23 am</t>
+  </si>
+  <si>
+    <t>king</t>
+  </si>
+  <si>
+    <t>king@gmail.com</t>
+  </si>
+  <si>
+    <t>9758468459</t>
+  </si>
+  <si>
+    <t>testing</t>
+  </si>
+  <si>
+    <t>7/6/2026, 12:45:18 am</t>
+  </si>
+  <si>
+    <t>hinmk</t>
+  </si>
+  <si>
+    <t>hinkk@gmail.com</t>
+  </si>
+  <si>
+    <t>9451236545</t>
+  </si>
+  <si>
+    <t>enquiry01</t>
+  </si>
+  <si>
+    <t>7/6/2026, 12:50:10 am</t>
   </si>
 </sst>
 </file>
@@ -676,7 +706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1234,6 +1264,70 @@
         <v>92</v>
       </c>
     </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" t="s">
+        <v>95</v>
+      </c>
+      <c r="E18" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" t="s">
+        <v>96</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" t="s">
+        <v>17</v>
+      </c>
+      <c r="J18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" t="s">
+        <v>100</v>
+      </c>
+      <c r="E19" t="s">
+        <v>29</v>
+      </c>
+      <c r="F19" t="s">
+        <v>101</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" t="s">
+        <v>17</v>
+      </c>
+      <c r="J19" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>